<commit_message>
release(beta): certify Strategic Fleet Manager Beta 1.0
- Complete Golden Fleet certification
- Basher and Shiv integrated
- Image registry certified
- Component catalog updated
- RC-001 through RC-001A complete
- Beta Release Candidate approved

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data-maintenance/ship-images/Commander RSI URL Master.xlsx
+++ b/data-maintenance/ship-images/Commander RSI URL Master.xlsx
@@ -1,17 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr/>
+  <bookViews>
+    <workbookView xWindow="510" yWindow="570" windowWidth="50535" windowHeight="19605"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="498" uniqueCount="498">
   <si>
     <t>100i</t>
   </si>
@@ -229,9 +232,6 @@
     <t>https://robertsspaceindustries.com/i/42b74db93a9d6c96407a15009a7f59c5f6faa6b6/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReseukDF2naM9B1uvYiDLtHy9cckjh49ysQA)/source.webp</t>
   </si>
   <si>
-    <t>Basher</t>
-  </si>
-  <si>
     <t>https://robertsspaceindustries.com/i/0b9fe8e5f747566daf22edfd015122cb496ea3c0/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjGhFzCnTPqyCWJEeaDBNB3oWvoHiUuXfc)/source.webp</t>
   </si>
   <si>
@@ -1129,9 +1129,6 @@
     <t>https://robertsspaceindustries.com/i/7f1723a830cbecad82904c64c92b272f397d341a/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjZuSweHytgpsb4fc3t87L1mXJcMGCCVF4)/source.webp</t>
   </si>
   <si>
-    <t>Shiv</t>
-  </si>
-  <si>
     <t>https://robertsspaceindustries.com/i/83496eb7312353e165beff60ddab7e534950beee/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReskfNjJxzLeJBQNwz8hZnHvXvcMscGngw4S)/source.webp</t>
   </si>
   <si>
@@ -1337,31 +1334,224 @@
   </si>
   <si>
     <t>https://robertsspaceindustries.com/i/201b16305598b3f101d78f2cf0f3bbeea5c5fd5f/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResivuuXPahoRKgQLW5h1aBypfa8P8Hap7Zg)/source.webp</t>
+  </si>
+  <si>
+    <t>Arrastra</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/75f93aebd4a3993b505cab5952c3a2612d246615/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReskGqWRY5r2ETXGZ1pbf58H16PhoeqWKwgS)/source.webp</t>
+  </si>
+  <si>
+    <t>Crucible</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/415207b24baccbc8f9a292682fbdf01419ed3c97/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResk6HKtm3JvRDjnuPsnSY6b1Tac2Ltkg4Tp)/source.webp</t>
+  </si>
+  <si>
+    <t>Endeavor</t>
+  </si>
+  <si>
+    <t>Expanse</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/3735ad32fa243c41350ff250ff3bbd5a15ca389a/resize(1820,1024,cover,hgjbks2vRxvijgZCkcudyey3yf2YnBqfanX6U636vzzNeeFdx43A2FpB2VsDZB7YNvCzEcXVwpZLUh2qptqc3g5fzN)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/741ef4cf2e3afdb9594b2361c4b9c383b89b0829/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReskfAiwB65NCsLfMiNpnNGtH6fJUffaK33C)/source.webp</t>
+  </si>
+  <si>
+    <t>G12</t>
+  </si>
+  <si>
+    <t>G12a</t>
+  </si>
+  <si>
+    <t>G12r</t>
+  </si>
+  <si>
+    <t>Galaxy</t>
+  </si>
+  <si>
+    <t>Genesis</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/c1db72ea5664129382c5835e60bece68e7047abc/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResikAxDJUFaGehK6AA3NYU2s6ocp5a3bykz)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/1900910628c5d39c4f6c8a2c98cb3223cd708ce3/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReseN3PD8Yei2EPy6cS9ZnRcMmF7kF9ZRb9G)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/7986dafd43313011d56deb6245f9a1dd756a5c7a/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjvy3bk4wqGTGYsbQr7UYYhqMXUFWU2se6)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/a4272169cfb07660d1e6045b23bd1789d8ff6acf/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResiirESnMrW6D9fAWNtn3qYqRC1e4x1yMUS)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/28b84eece3d88da1ef46512f5ccda2d52ab5188b/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjCZtmWTXGYC6ppEv2dfyqgTt8K3kv8r4E)/source.webp</t>
+  </si>
+  <si>
+    <t>Hull D</t>
+  </si>
+  <si>
+    <t>Hull E</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/195af2372d8b1f5c8468458a6e8fa1aedf2b9a50/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReseGuzyu4pRpM27n6RHhMau4SpgRfZtrpLe)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/e508950f37c0962bfa3a86bbee2a49b4af2a815c/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjYX8AoSzGvZWyXisKXvXGrmWWbFuRCfuG)/source.webp</t>
+  </si>
+  <si>
+    <t>Javelin</t>
+  </si>
+  <si>
+    <t>Kraken</t>
+  </si>
+  <si>
+    <t>Kraken Privateer</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/d06d02ee0e01ad6dcb16561795ae4cd8f87186a3/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjvbX42c3rKWbDaqUyqNmKE6rWyf9aufLJ)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/cb1e6580add474b7f3f2bf18f5081326d5967779/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjqYHRGgyn5CBWsSTK3b9eZJ6fQD1C1ydp)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/7bdbb6f6645c025a35597d000693eefe0b1266bf/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjqYJiA954ovGyjrhJzKDcRSB3GeX5S1Wn)/source.webp</t>
+  </si>
+  <si>
+    <t>Legionnaire</t>
+  </si>
+  <si>
+    <t>Liberator</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/2c603af2f1cf33d18fdb74cba906b0f3e45b2e8e/resize(1820,1024,cover,hgjbks2vRxvijgZCkcudyey3yf2YnBqfanX6U636vzzNeeFdx43A2FpAyJAaJtycCHer7whEazSZzqQ1QuY25bU1DQ)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/eed7bda0cead13f22d29e0e4898532db163e4fae/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjYSRgY9JUi324WZvNLjX8bNV6rD8Rtger)/source.webp</t>
+  </si>
+  <si>
+    <t>Merchantman</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/322572eafa4b6dbc3c2c540549793c5bf9b23168/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjCWNfq9LLyC3dvte2ieQJwYuocquD6xva)/source.webp</t>
+  </si>
+  <si>
+    <t>Nautilus</t>
+  </si>
+  <si>
+    <t>Nautilus Solstice Edition</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/051670c059dacd122a5d9fb45b10f9471a5aab80/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResipDnNrrrz7nbvL1DVJLNr6dYAYCQ3zryk)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/722e3fae113bff8da25fdc1548364efb6dcde748/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResjkHkFivXFNwMzRH2zpNDhn2HKZyoE4MCJ)/source.webp</t>
+  </si>
+  <si>
+    <t>Odin</t>
+  </si>
+  <si>
+    <t>Odyssey</t>
+  </si>
+  <si>
+    <t>Orion</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/8249f977d844d3f51435259d4e4c4cb7b874c547/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResivtfLYvFyzwfYeFzw5w3FpCeXVUZoNytJ)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/ccf8090a7f5107857af3115ac8535c25ac486d30/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReskkTUwu7hSxftmz1nsS3kx4Xi3ZuZQfPug)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/bed5c9e3b6d417d3056b6dabf8f37ef6dca64232/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResiisVBYsvtdRnA1UfqpGr22gNgMyVa6hVQ)/source.webp</t>
+  </si>
+  <si>
+    <t>Pioneer</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/50bb5d2f215ab21fc4d13bb241c001c64cb33eaa/resize(1820,1024,cover,hgjbks2vRxvijgZCkcudyey3yf2YnBqfanX6U636vzzNeeFdx43A2FpB1JVc7Xvq4q8CRfEHpFzSVmnzxaoM65fTo4)/source.webp</t>
+  </si>
+  <si>
+    <t>Ranger CV</t>
+  </si>
+  <si>
+    <t>Ranger RC</t>
+  </si>
+  <si>
+    <t>Ranger TR</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/cb9372a344546093df8cad357d8a536f8b68411d/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjReseH3Qd7shCav1BWchG74sQDq23zWLm3txN)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/b0d508d728dd6d858f390710450e9c1cfb35af25/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResetri3LoJRN1ys3QbytxFzJtbwr53ABJ62)/source.webp</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/66f8e7da7717c6b3aa1522b9cabd0b267142cbdb/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResj1mPB5zoigCCxoe5NAe8g6Ak9JAjpms7t)/source.webp</t>
+  </si>
+  <si>
+    <t>Vulcan</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/9e7e9b7b18f90777c9ab34b571dbacf470d78c52/resize(1820,1024,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResejVm2oahKQbxntDyDipVCaX4byAbDNp6a)/source.webp</t>
+  </si>
+  <si>
+    <t>Zeus Mk II MR</t>
+  </si>
+  <si>
+    <t>https://robertsspaceindustries.com/i/d0d0aa31e84898d35f276ab65174a292509f9db4/resize(910,512,cover,ADdPNihJzmPbNuTnFsH1DqUeqBRpXdSXVVtgJTyDDgscGKrzJuoFjResk22Znp2LVdS2JMxJFjrYCirRpVc4v9Pzv)/source.webp</t>
+  </si>
+  <si>
+    <t>Grey's Basher</t>
+  </si>
+  <si>
+    <t>Grey's Shiv</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1369,38 +1559,42 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+  <cellStyleXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1408,7 +1602,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1598,21 +1792,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:B249"/>
+  <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="25.5"/>
-    <col customWidth="1" min="2" max="2" width="195.13"/>
+    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="2" max="2" width="215.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1620,7 +1817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -1628,7 +1825,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -1636,7 +1833,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1644,7 +1841,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
@@ -1652,7 +1849,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -1660,7 +1857,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
@@ -1668,7 +1865,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
@@ -1676,7 +1873,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>16</v>
       </c>
@@ -1684,7 +1881,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
@@ -1692,7 +1889,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -1700,7 +1897,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
@@ -1708,7 +1905,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -1716,7 +1913,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
@@ -1724,7 +1921,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
@@ -1732,7 +1929,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>30</v>
       </c>
@@ -1740,7 +1937,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>32</v>
       </c>
@@ -1748,7 +1945,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>34</v>
       </c>
@@ -1756,1854 +1953,2080 @@
         <v>35</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
+        <v>440</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A20" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="1" t="s">
+    <row r="21" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A21" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B21" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="1" t="s">
+    <row r="22" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B22" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="1" t="s">
+    <row r="23" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A23" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B23" s="2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A24" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B24" s="2" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="1" t="s">
+    <row r="25" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A25" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B25" s="2" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="1" t="s">
+    <row r="26" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A26" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B26" s="2" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A27" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B27" s="2" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="1" t="s">
+    <row r="28" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A28" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B28" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="s">
+    <row r="29" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B29" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="1" t="s">
+    <row r="30" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B29" s="2" t="s">
+      <c r="B30" s="2" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="1" t="s">
+    <row r="31" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B31" s="3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="1" t="s">
+    <row r="32" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A32" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B32" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="1" t="s">
+    <row r="33" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A33" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B33" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A34" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B34" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="1" t="s">
+    <row r="35" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A35" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="B35" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="1" t="s">
+    <row r="36" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A36" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B36" s="3" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="1" t="s">
+    <row r="37" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A37" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="B37" s="3" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="s">
+    <row r="38" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A38" s="1" t="s">
+        <v>496</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B37" s="2" t="s">
+    </row>
+    <row r="39" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="s">
+      <c r="B39" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B38" s="2" t="s">
+    </row>
+    <row r="40" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A40" s="1" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="s">
+      <c r="B40" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="B39" s="2" t="s">
+    </row>
+    <row r="41" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A41" s="1" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="s">
+      <c r="B41" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B40" s="3" t="s">
+    </row>
+    <row r="42" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A42" s="1" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="s">
+      <c r="B42" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B41" s="3" t="s">
+    </row>
+    <row r="43" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="s">
+      <c r="B43" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B42" s="2" t="s">
+    </row>
+    <row r="44" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
         <v>83</v>
       </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="s">
+      <c r="B44" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B43" s="3" t="s">
+    </row>
+    <row r="45" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="s">
+      <c r="B45" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B44" s="3" t="s">
+    </row>
+    <row r="46" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A46" s="1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="s">
+      <c r="B46" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B45" s="3" t="s">
+    </row>
+    <row r="47" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A47" s="1" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="1" t="s">
+      <c r="B47" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B46" s="3" t="s">
+    </row>
+    <row r="48" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A48" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="1" t="s">
+      <c r="B48" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B47" s="3" t="s">
+    </row>
+    <row r="49" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A49" s="1" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="1" t="s">
+      <c r="B49" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="B48" s="3" t="s">
+    </row>
+    <row r="50" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A50" s="1" t="s">
         <v>95</v>
       </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="1" t="s">
+      <c r="B50" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B49" s="3" t="s">
+    </row>
+    <row r="51" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A51" s="1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="1" t="s">
+      <c r="B51" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B50" s="3" t="s">
+    </row>
+    <row r="52" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A52" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="1" t="s">
+      <c r="B52" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B51" s="3" t="s">
+    </row>
+    <row r="53" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A53" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="1" t="s">
+      <c r="B53" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B52" s="3" t="s">
+    </row>
+    <row r="54" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A54" s="1" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="s">
+      <c r="B54" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B53" s="3" t="s">
+    </row>
+    <row r="55" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A55" s="1" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="s">
+      <c r="B55" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B54" s="3" t="s">
+    </row>
+    <row r="56" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="s">
+      <c r="B56" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B55" s="3" t="s">
+    </row>
+    <row r="57" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>442</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="s">
+      <c r="B58" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B56" s="3" t="s">
+    </row>
+    <row r="59" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A59" s="1" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="s">
+      <c r="B59" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="B57" s="3" t="s">
+    </row>
+    <row r="60" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A60" s="1" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="s">
+      <c r="B60" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B58" s="3" t="s">
+    </row>
+    <row r="61" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A61" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="s">
+      <c r="B61" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="B59" s="3" t="s">
+    </row>
+    <row r="62" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A62" s="1" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="s">
+      <c r="B62" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="B60" s="3" t="s">
+    </row>
+    <row r="63" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A63" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="s">
+      <c r="B63" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B61" s="3" t="s">
+    </row>
+    <row r="64" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A64" s="1" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="s">
+      <c r="B64" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="B62" s="3" t="s">
+    </row>
+    <row r="65" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A65" s="1" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="s">
+      <c r="B65" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="B63" s="3" t="s">
+    </row>
+    <row r="66" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A66" s="1" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="1" t="s">
+      <c r="B66" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B64" s="3" t="s">
+    </row>
+    <row r="67" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A67" s="1" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="1" t="s">
+      <c r="B67" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="B65" s="3" t="s">
+    </row>
+    <row r="68" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A68" s="1" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="1" t="s">
+      <c r="B68" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="B66" s="3" t="s">
+    </row>
+    <row r="69" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A69" s="1" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="1" t="s">
+      <c r="B69" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B67" s="3" t="s">
+    </row>
+    <row r="70" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A70" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="1" t="s">
+      <c r="B70" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B68" s="3" t="s">
+    </row>
+    <row r="71" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A71" s="1" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="1" t="s">
+      <c r="B71" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B69" s="3" t="s">
+    </row>
+    <row r="72" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A72" s="1" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="s">
+      <c r="B72" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B70" s="3" t="s">
+    </row>
+    <row r="73" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A73" s="1" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="1" t="s">
+      <c r="B73" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B71" s="3" t="s">
+    </row>
+    <row r="74" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A74" s="1" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="s">
+      <c r="B74" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="B72" s="3" t="s">
+    </row>
+    <row r="75" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A75" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="s">
+      <c r="B75" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="B73" s="3" t="s">
+    </row>
+    <row r="76" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A76" s="1" t="s">
+        <v>444</v>
+      </c>
+      <c r="B76" s="3" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A77" s="1" t="s">
+        <v>445</v>
+      </c>
+      <c r="B77" s="3" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A78" s="1" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="1" t="s">
+      <c r="B78" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B74" s="3" t="s">
+    </row>
+    <row r="79" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A79" s="1" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="s">
+      <c r="B79" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B75" s="3" t="s">
+    </row>
+    <row r="80" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A80" s="1" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="1" t="s">
+      <c r="B80" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B76" s="3" t="s">
+    </row>
+    <row r="81" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A81" s="1" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="1" t="s">
+      <c r="B81" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="B77" s="3" t="s">
+    </row>
+    <row r="82" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A82" s="1" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="1" t="s">
+      <c r="B82" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="B78" s="3" t="s">
+    </row>
+    <row r="83" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A83" s="1" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="1" t="s">
+      <c r="B83" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="B79" s="2" t="s">
+    </row>
+    <row r="84" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A84" s="1" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="1" t="s">
+      <c r="B84" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="B80" s="3" t="s">
+    </row>
+    <row r="85" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A85" s="1" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="1" t="s">
+      <c r="B85" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="B81" s="3" t="s">
+    </row>
+    <row r="86" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A86" s="1" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="1" t="s">
+      <c r="B86" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="B82" s="3" t="s">
+    </row>
+    <row r="87" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A87" s="1" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="1" t="s">
+      <c r="B87" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="B83" s="3" t="s">
+    </row>
+    <row r="88" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A88" s="1" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="1" t="s">
+      <c r="B88" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B84" s="3" t="s">
+    </row>
+    <row r="89" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A89" s="1" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="1" t="s">
+      <c r="B89" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="B85" s="3" t="s">
+    </row>
+    <row r="90" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A90" s="1" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="1" t="s">
+      <c r="B90" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="B86" s="3" t="s">
+    </row>
+    <row r="91" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A91" s="1" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="1" t="s">
+      <c r="B91" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="B87" s="3" t="s">
+    </row>
+    <row r="92" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A92" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="1" t="s">
+      <c r="B92" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="B88" s="3" t="s">
+    </row>
+    <row r="93" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A93" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="1" t="s">
+      <c r="B93" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="B89" s="3" t="s">
+    </row>
+    <row r="94" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A94" s="1" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="1" t="s">
+      <c r="B94" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="B90" s="3" t="s">
+    </row>
+    <row r="95" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A95" s="1" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="1" t="s">
+      <c r="B95" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="B91" s="3" t="s">
+    </row>
+    <row r="96" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A96" s="1" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="1" t="s">
+      <c r="B96" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="B92" s="3" t="s">
+    </row>
+    <row r="97" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A97" s="1" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="1" t="s">
+      <c r="B97" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="B93" s="3" t="s">
+    </row>
+    <row r="98" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A98" s="1" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="1" t="s">
+      <c r="B98" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="B94" s="3" t="s">
+    </row>
+    <row r="99" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A99" s="1" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1" t="s">
+      <c r="B99" s="3" t="s">
         <v>188</v>
       </c>
-      <c r="B95" s="3" t="s">
+    </row>
+    <row r="100" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A100" s="1" t="s">
+        <v>448</v>
+      </c>
+      <c r="B100" s="3" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A101" s="1" t="s">
+        <v>449</v>
+      </c>
+      <c r="B101" s="3" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A102" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="B102" s="3" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A103" s="1" t="s">
+        <v>451</v>
+      </c>
+      <c r="B103" s="3" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A104" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A105" s="1" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="1" t="s">
+      <c r="B105" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="B96" s="3" t="s">
+    </row>
+    <row r="106" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A106" s="1" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="1" t="s">
+      <c r="B106" s="3" t="s">
         <v>192</v>
       </c>
-      <c r="B97" s="3" t="s">
+    </row>
+    <row r="107" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A107" s="1" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="1" t="s">
+      <c r="B107" s="3" t="s">
         <v>194</v>
       </c>
-      <c r="B98" s="3" t="s">
+    </row>
+    <row r="108" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A108" s="1" t="s">
         <v>195</v>
       </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="1" t="s">
+      <c r="B108" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="B99" s="3" t="s">
+    </row>
+    <row r="109" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A109" s="1" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="1" t="s">
+      <c r="B109" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="B100" s="3" t="s">
+    </row>
+    <row r="110" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A110" s="1" t="s">
         <v>199</v>
       </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="1" t="s">
+      <c r="B110" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="B101" s="3" t="s">
+    </row>
+    <row r="111" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A111" s="1" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="1" t="s">
+      <c r="B111" s="3" t="s">
         <v>202</v>
       </c>
-      <c r="B102" s="3" t="s">
+    </row>
+    <row r="112" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A112" s="1" t="s">
         <v>203</v>
       </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="1" t="s">
+      <c r="B112" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="B103" s="3" t="s">
+    </row>
+    <row r="113" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A113" s="1" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="1" t="s">
+      <c r="B113" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B104" s="3" t="s">
+    </row>
+    <row r="114" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A114" s="1" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="1" t="s">
+      <c r="B114" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="B105" s="3" t="s">
+    </row>
+    <row r="115" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A115" s="1" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="1" t="s">
+      <c r="B115" s="3" t="s">
         <v>210</v>
       </c>
-      <c r="B106" s="3" t="s">
+    </row>
+    <row r="116" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A116" s="1" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="1" t="s">
+      <c r="B116" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="B107" s="3" t="s">
+    </row>
+    <row r="117" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A117" s="1" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="1" t="s">
+      <c r="B117" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="B108" s="3" t="s">
+    </row>
+    <row r="118" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A118" s="1" t="s">
         <v>215</v>
       </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="s">
+      <c r="B118" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="B109" s="3" t="s">
+    </row>
+    <row r="119" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A119" s="1" t="s">
         <v>217</v>
       </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="s">
+      <c r="B119" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B110" s="3" t="s">
+    </row>
+    <row r="120" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A120" s="1" t="s">
         <v>219</v>
       </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="s">
+      <c r="B120" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="B111" s="3" t="s">
+    </row>
+    <row r="121" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A121" s="1" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="s">
+      <c r="B121" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B112" s="3" t="s">
+    </row>
+    <row r="122" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A122" s="1" t="s">
         <v>223</v>
       </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="1" t="s">
+      <c r="B122" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B113" s="3" t="s">
+    </row>
+    <row r="123" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A123" s="1" t="s">
+        <v>458</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A124" s="1" t="s">
+        <v>459</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A125" s="1" t="s">
         <v>225</v>
       </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="1" t="s">
+      <c r="B125" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="B114" s="3" t="s">
+    </row>
+    <row r="126" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A126" s="1" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="1" t="s">
+      <c r="B126" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="B115" s="3" t="s">
+    </row>
+    <row r="127" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A127" s="1" t="s">
         <v>229</v>
       </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="1" t="s">
+      <c r="B127" s="3" t="s">
         <v>230</v>
       </c>
-      <c r="B116" s="3" t="s">
+    </row>
+    <row r="128" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A128" s="1" t="s">
         <v>231</v>
       </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="1" t="s">
+      <c r="B128" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B117" s="3" t="s">
+    </row>
+    <row r="129" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A129" s="1" t="s">
         <v>233</v>
       </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="1" t="s">
+      <c r="B129" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="B118" s="3" t="s">
+    </row>
+    <row r="130" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A130" s="1" t="s">
         <v>235</v>
       </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="1" t="s">
+      <c r="B130" s="3" t="s">
         <v>236</v>
       </c>
-      <c r="B119" s="3" t="s">
+    </row>
+    <row r="131" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A131" s="1" t="s">
+        <v>462</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A132" s="1" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="1" t="s">
+      <c r="B132" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="B120" s="3" t="s">
+    </row>
+    <row r="133" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A133" s="1" t="s">
+        <v>463</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A134" s="1" t="s">
+        <v>464</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A135" s="1" t="s">
         <v>239</v>
       </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="1" t="s">
+      <c r="B135" s="3" t="s">
         <v>240</v>
       </c>
-      <c r="B121" s="3" t="s">
+    </row>
+    <row r="136" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A136" s="1" t="s">
         <v>241</v>
       </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="1" t="s">
+      <c r="B136" s="3" t="s">
         <v>242</v>
       </c>
-      <c r="B122" s="3" t="s">
+    </row>
+    <row r="137" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A137" s="1" t="s">
+        <v>468</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A138" s="1" t="s">
+        <v>469</v>
+      </c>
+      <c r="B138" s="3" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A139" s="1" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="1" t="s">
+      <c r="B139" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="B123" s="3" t="s">
+    </row>
+    <row r="140" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A140" s="1" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="1" t="s">
+      <c r="B140" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="B124" s="3" t="s">
+    </row>
+    <row r="141" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A141" s="1" t="s">
         <v>247</v>
       </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="1" t="s">
+      <c r="B141" s="3" t="s">
         <v>248</v>
       </c>
-      <c r="B125" s="3" t="s">
+    </row>
+    <row r="142" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A142" s="1" t="s">
         <v>249</v>
       </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="1" t="s">
+      <c r="B142" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="B126" s="3" t="s">
+    </row>
+    <row r="143" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A143" s="1" t="s">
         <v>251</v>
       </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="1" t="s">
+      <c r="B143" s="3" t="s">
         <v>252</v>
       </c>
-      <c r="B127" s="3" t="s">
+    </row>
+    <row r="144" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A144" s="1" t="s">
         <v>253</v>
       </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="1" t="s">
+      <c r="B144" s="3" t="s">
         <v>254</v>
       </c>
-      <c r="B128" s="3" t="s">
+    </row>
+    <row r="145" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A145" s="1" t="s">
+        <v>472</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A146" s="1" t="s">
         <v>255</v>
       </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="1" t="s">
+      <c r="B146" s="3" t="s">
         <v>256</v>
       </c>
-      <c r="B129" s="3" t="s">
+    </row>
+    <row r="147" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A147" s="1" t="s">
         <v>257</v>
       </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="1" t="s">
+      <c r="B147" s="3" t="s">
         <v>258</v>
       </c>
-      <c r="B130" s="3" t="s">
+    </row>
+    <row r="148" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A148" s="1" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="1" t="s">
+      <c r="B148" s="3" t="s">
         <v>260</v>
       </c>
-      <c r="B131" s="3" t="s">
+    </row>
+    <row r="149" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A149" s="1" t="s">
         <v>261</v>
       </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="1" t="s">
+      <c r="B149" s="3" t="s">
         <v>262</v>
       </c>
-      <c r="B132" s="3" t="s">
+    </row>
+    <row r="150" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A150" s="1" t="s">
         <v>263</v>
       </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="1" t="s">
+      <c r="B150" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="B133" s="3" t="s">
+    </row>
+    <row r="151" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A151" s="1" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="1" t="s">
+      <c r="B151" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="B134" s="3" t="s">
+    </row>
+    <row r="152" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A152" s="1" t="s">
         <v>267</v>
       </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="1" t="s">
+      <c r="B152" s="3" t="s">
         <v>268</v>
       </c>
-      <c r="B135" s="3" t="s">
+    </row>
+    <row r="153" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A153" s="1" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="1" t="s">
+      <c r="B153" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="B136" s="3" t="s">
+    </row>
+    <row r="154" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A154" s="1" t="s">
         <v>271</v>
       </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="1" t="s">
+      <c r="B154" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="B137" s="3" t="s">
+    </row>
+    <row r="155" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A155" s="1" t="s">
         <v>273</v>
       </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="1" t="s">
+      <c r="B155" s="3" t="s">
         <v>274</v>
       </c>
-      <c r="B138" s="3" t="s">
+    </row>
+    <row r="156" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A156" s="1" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="139">
-      <c r="A139" s="1" t="s">
+      <c r="B156" s="3" t="s">
         <v>276</v>
       </c>
-      <c r="B139" s="3" t="s">
+    </row>
+    <row r="157" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A157" s="1" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="1" t="s">
+      <c r="B157" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="B140" s="3" t="s">
+    </row>
+    <row r="158" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A158" s="1" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="1" t="s">
+      <c r="B158" s="3" t="s">
         <v>280</v>
       </c>
-      <c r="B141" s="3" t="s">
+    </row>
+    <row r="159" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A159" s="1" t="s">
         <v>281</v>
       </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="1" t="s">
+      <c r="B159" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="B142" s="3" t="s">
+    </row>
+    <row r="160" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A160" s="1" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="143">
-      <c r="A143" s="1" t="s">
+      <c r="B160" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="B143" s="3" t="s">
+    </row>
+    <row r="161" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A161" s="1" t="s">
         <v>285</v>
       </c>
-    </row>
-    <row r="144">
-      <c r="A144" s="1" t="s">
+      <c r="B161" s="3" t="s">
         <v>286</v>
       </c>
-      <c r="B144" s="3" t="s">
+    </row>
+    <row r="162" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A162" s="1" t="s">
         <v>287</v>
       </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="1" t="s">
+      <c r="B162" s="3" t="s">
         <v>288</v>
       </c>
-      <c r="B145" s="3" t="s">
+    </row>
+    <row r="163" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A163" s="1" t="s">
+        <v>474</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A164" s="1" t="s">
+        <v>475</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A165" s="1" t="s">
         <v>289</v>
       </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="1" t="s">
+      <c r="B165" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="B146" s="3" t="s">
+    </row>
+    <row r="166" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A166" s="1" t="s">
         <v>291</v>
       </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="1" t="s">
+      <c r="B166" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="B147" s="3" t="s">
+    </row>
+    <row r="167" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A167" s="1" t="s">
         <v>293</v>
       </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="1" t="s">
+      <c r="B167" s="3" t="s">
         <v>294</v>
       </c>
-      <c r="B148" s="3" t="s">
+    </row>
+    <row r="168" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A168" s="1" t="s">
         <v>295</v>
       </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="1" t="s">
+      <c r="B168" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="B149" s="3" t="s">
+    </row>
+    <row r="169" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A169" s="1" t="s">
+        <v>478</v>
+      </c>
+      <c r="B169" s="3" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A170" s="1" t="s">
+        <v>479</v>
+      </c>
+      <c r="B170" s="3" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="171" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A171" s="1" t="s">
+        <v>480</v>
+      </c>
+      <c r="B171" s="3" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="172" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A172" s="1" t="s">
         <v>297</v>
       </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="1" t="s">
+      <c r="B172" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="B150" s="3" t="s">
+    </row>
+    <row r="173" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A173" s="1" t="s">
         <v>299</v>
       </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="1" t="s">
+      <c r="B173" s="3" t="s">
         <v>300</v>
       </c>
-      <c r="B151" s="3" t="s">
+    </row>
+    <row r="174" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A174" s="1" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="1" t="s">
+      <c r="B174" s="3" t="s">
         <v>302</v>
       </c>
-      <c r="B152" s="3" t="s">
+    </row>
+    <row r="175" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A175" s="1" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="1" t="s">
+      <c r="B175" s="3" t="s">
         <v>304</v>
       </c>
-      <c r="B153" s="3" t="s">
+    </row>
+    <row r="176" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A176" s="1" t="s">
         <v>305</v>
       </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="1" t="s">
+      <c r="B176" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="B154" s="3" t="s">
+    </row>
+    <row r="177" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A177" s="1" t="s">
+        <v>484</v>
+      </c>
+      <c r="B177" s="3" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="178" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A178" s="1" t="s">
         <v>307</v>
       </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="1" t="s">
+      <c r="B178" s="3" t="s">
         <v>308</v>
       </c>
-      <c r="B155" s="3" t="s">
+    </row>
+    <row r="179" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A179" s="1" t="s">
         <v>309</v>
       </c>
-    </row>
-    <row r="156">
-      <c r="A156" s="1" t="s">
+      <c r="B179" s="3" t="s">
         <v>310</v>
       </c>
-      <c r="B156" s="3" t="s">
+    </row>
+    <row r="180" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A180" s="1" t="s">
         <v>311</v>
       </c>
-    </row>
-    <row r="157">
-      <c r="A157" s="1" t="s">
+      <c r="B180" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="B157" s="3" t="s">
+    </row>
+    <row r="181" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A181" s="1" t="s">
         <v>313</v>
       </c>
-    </row>
-    <row r="158">
-      <c r="A158" s="1" t="s">
+      <c r="B181" s="3" t="s">
         <v>314</v>
       </c>
-      <c r="B158" s="3" t="s">
+    </row>
+    <row r="182" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A182" s="1" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="159">
-      <c r="A159" s="1" t="s">
+      <c r="B182" s="3" t="s">
         <v>316</v>
       </c>
-      <c r="B159" s="3" t="s">
+    </row>
+    <row r="183" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A183" s="1" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="160">
-      <c r="A160" s="1" t="s">
+      <c r="B183" s="3" t="s">
         <v>318</v>
       </c>
-      <c r="B160" s="3" t="s">
+    </row>
+    <row r="184" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A184" s="1" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="161">
-      <c r="A161" s="1" t="s">
+      <c r="B184" s="3" t="s">
         <v>320</v>
       </c>
-      <c r="B161" s="3" t="s">
+    </row>
+    <row r="185" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A185" s="1" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="162">
-      <c r="A162" s="1" t="s">
+      <c r="B185" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="B162" s="3" t="s">
+    </row>
+    <row r="186" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A186" s="1" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="163">
-      <c r="A163" s="1" t="s">
+      <c r="B186" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="B163" s="3" t="s">
+    </row>
+    <row r="187" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A187" s="1" t="s">
         <v>325</v>
       </c>
-    </row>
-    <row r="164">
-      <c r="A164" s="1" t="s">
+      <c r="B187" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="B164" s="3" t="s">
+    </row>
+    <row r="188" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A188" s="1" t="s">
+        <v>486</v>
+      </c>
+      <c r="B188" s="3" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="189" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A189" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B189" s="3" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="190" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A190" s="1" t="s">
+        <v>488</v>
+      </c>
+      <c r="B190" s="3" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="191" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A191" s="1" t="s">
         <v>327</v>
       </c>
-    </row>
-    <row r="165">
-      <c r="A165" s="1" t="s">
+      <c r="B191" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="B165" s="3" t="s">
+    </row>
+    <row r="192" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A192" s="1" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="166">
-      <c r="A166" s="1" t="s">
+      <c r="B192" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B166" s="3" t="s">
+    </row>
+    <row r="193" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A193" s="1" t="s">
         <v>331</v>
       </c>
-    </row>
-    <row r="167">
-      <c r="A167" s="1" t="s">
+      <c r="B193" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="B167" s="3" t="s">
+    </row>
+    <row r="194" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A194" s="1" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="168">
-      <c r="A168" s="1" t="s">
+      <c r="B194" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="B168" s="3" t="s">
+    </row>
+    <row r="195" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A195" s="1" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="169">
-      <c r="A169" s="1" t="s">
+      <c r="B195" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="B169" s="3" t="s">
+    </row>
+    <row r="196" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A196" s="1" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="1" t="s">
+      <c r="B196" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="B170" s="3" t="s">
+    </row>
+    <row r="197" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A197" s="1" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="1" t="s">
+      <c r="B197" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="B171" s="3" t="s">
+    </row>
+    <row r="198" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A198" s="1" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="1" t="s">
+      <c r="B198" s="3" t="s">
         <v>342</v>
       </c>
-      <c r="B172" s="3" t="s">
+    </row>
+    <row r="199" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A199" s="1" t="s">
         <v>343</v>
       </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="1" t="s">
+      <c r="B199" s="3" t="s">
         <v>344</v>
       </c>
-      <c r="B173" s="3" t="s">
+    </row>
+    <row r="200" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A200" s="1" t="s">
         <v>345</v>
       </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="1" t="s">
+      <c r="B200" s="3" t="s">
         <v>346</v>
       </c>
-      <c r="B174" s="3" t="s">
+    </row>
+    <row r="201" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A201" s="1" t="s">
         <v>347</v>
       </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="1" t="s">
+      <c r="B201" s="3" t="s">
         <v>348</v>
       </c>
-      <c r="B175" s="3" t="s">
+    </row>
+    <row r="202" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A202" s="1" t="s">
         <v>349</v>
       </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="1" t="s">
+      <c r="B202" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="B176" s="3" t="s">
+    </row>
+    <row r="203" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A203" s="1" t="s">
         <v>351</v>
       </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="1" t="s">
+      <c r="B203" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="B177" s="3" t="s">
+    </row>
+    <row r="204" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A204" s="1" t="s">
         <v>353</v>
       </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="1" t="s">
+      <c r="B204" s="3" t="s">
         <v>354</v>
       </c>
-      <c r="B178" s="3" t="s">
+    </row>
+    <row r="205" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A205" s="1" t="s">
         <v>355</v>
       </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="1" t="s">
+      <c r="B205" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="B179" s="3" t="s">
+    </row>
+    <row r="206" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A206" s="1" t="s">
         <v>357</v>
       </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="1" t="s">
+      <c r="B206" s="3" t="s">
         <v>358</v>
       </c>
-      <c r="B180" s="3" t="s">
+    </row>
+    <row r="207" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A207" s="1" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="1" t="s">
+      <c r="B207" s="3" t="s">
         <v>360</v>
       </c>
-      <c r="B181" s="3" t="s">
+    </row>
+    <row r="208" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A208" s="1" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="1" t="s">
+      <c r="B208" s="3" t="s">
         <v>362</v>
       </c>
-      <c r="B182" s="3" t="s">
+    </row>
+    <row r="209" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A209" s="1" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="1" t="s">
+      <c r="B209" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="B183" s="3" t="s">
+    </row>
+    <row r="210" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A210" s="1" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="1" t="s">
+      <c r="B210" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="B184" s="3" t="s">
+    </row>
+    <row r="211" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A211" s="1" t="s">
         <v>367</v>
       </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="1" t="s">
+      <c r="B211" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="B185" s="3" t="s">
+    </row>
+    <row r="212" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A212" s="1" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="1" t="s">
+      <c r="B212" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="B186" s="3" t="s">
+    </row>
+    <row r="213" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A213" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="B213" s="3" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="187">
-      <c r="A187" s="1" t="s">
+    <row r="214" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A214" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="B187" s="3" t="s">
+      <c r="B214" s="3" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="188">
-      <c r="A188" s="1" t="s">
+    <row r="215" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A215" s="1" t="s">
         <v>374</v>
       </c>
-      <c r="B188" s="3" t="s">
+      <c r="B215" s="3" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="189">
-      <c r="A189" s="1" t="s">
+    <row r="216" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A216" s="1" t="s">
         <v>376</v>
       </c>
-      <c r="B189" s="3" t="s">
+      <c r="B216" s="3" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="190">
-      <c r="A190" s="1" t="s">
+    <row r="217" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A217" s="1" t="s">
         <v>378</v>
       </c>
-      <c r="B190" s="3" t="s">
+      <c r="B217" s="3" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="191">
-      <c r="A191" s="1" t="s">
+    <row r="218" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A218" s="1" t="s">
         <v>380</v>
       </c>
-      <c r="B191" s="3" t="s">
+      <c r="B218" s="3" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="192">
-      <c r="A192" s="1" t="s">
+    <row r="219" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A219" s="1" t="s">
         <v>382</v>
       </c>
-      <c r="B192" s="3" t="s">
+      <c r="B219" s="3" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="193">
-      <c r="A193" s="1" t="s">
+    <row r="220" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A220" s="1" t="s">
         <v>384</v>
       </c>
-      <c r="B193" s="3" t="s">
+      <c r="B220" s="3" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="194">
-      <c r="A194" s="1" t="s">
+    <row r="221" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A221" s="1" t="s">
         <v>386</v>
       </c>
-      <c r="B194" s="3" t="s">
+      <c r="B221" s="3" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="195">
-      <c r="A195" s="1" t="s">
+    <row r="222" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A222" s="1" t="s">
         <v>388</v>
       </c>
-      <c r="B195" s="3" t="s">
+      <c r="B222" s="3" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="196">
-      <c r="A196" s="1" t="s">
+    <row r="223" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A223" s="1" t="s">
         <v>390</v>
       </c>
-      <c r="B196" s="3" t="s">
+      <c r="B223" s="3" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="1" t="s">
+    <row r="224" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A224" s="1" t="s">
         <v>392</v>
       </c>
-      <c r="B197" s="3" t="s">
+      <c r="B224" s="3" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="198">
-      <c r="A198" s="1" t="s">
+    <row r="225" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A225" s="1" t="s">
         <v>394</v>
       </c>
-      <c r="B198" s="3" t="s">
+      <c r="B225" s="3" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="199">
-      <c r="A199" s="1" t="s">
+    <row r="226" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A226" s="1" t="s">
         <v>396</v>
       </c>
-      <c r="B199" s="3" t="s">
+      <c r="B226" s="3" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="200">
-      <c r="A200" s="1" t="s">
+    <row r="227" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A227" s="1" t="s">
         <v>398</v>
       </c>
-      <c r="B200" s="3" t="s">
+      <c r="B227" s="3" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="201">
-      <c r="A201" s="1" t="s">
+    <row r="228" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A228" s="1" t="s">
         <v>400</v>
       </c>
-      <c r="B201" s="3" t="s">
+      <c r="B228" s="3" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="202">
-      <c r="A202" s="1" t="s">
+    <row r="229" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A229" s="1" t="s">
         <v>402</v>
       </c>
-      <c r="B202" s="3" t="s">
+      <c r="B229" s="3" t="s">
         <v>403</v>
       </c>
     </row>
-    <row r="203">
-      <c r="A203" s="1" t="s">
+    <row r="230" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A230" s="1" t="s">
         <v>404</v>
       </c>
-      <c r="B203" s="3" t="s">
+      <c r="B230" s="3" t="s">
         <v>405</v>
       </c>
     </row>
-    <row r="204">
-      <c r="A204" s="1" t="s">
+    <row r="231" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A231" s="1" t="s">
         <v>406</v>
       </c>
-      <c r="B204" s="3" t="s">
+      <c r="B231" s="3" t="s">
         <v>407</v>
       </c>
     </row>
-    <row r="205">
-      <c r="A205" s="1" t="s">
+    <row r="232" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A232" s="1" t="s">
         <v>408</v>
       </c>
-      <c r="B205" s="3" t="s">
+      <c r="B232" s="3" t="s">
         <v>409</v>
       </c>
     </row>
-    <row r="206">
-      <c r="A206" s="1" t="s">
+    <row r="233" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A233" s="1" t="s">
         <v>410</v>
       </c>
-      <c r="B206" s="3" t="s">
+      <c r="B233" s="3" t="s">
         <v>411</v>
       </c>
     </row>
-    <row r="207">
-      <c r="A207" s="1" t="s">
+    <row r="234" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A234" s="1" t="s">
         <v>412</v>
       </c>
-      <c r="B207" s="3" t="s">
+      <c r="B234" s="3" t="s">
         <v>413</v>
       </c>
     </row>
-    <row r="208">
-      <c r="A208" s="1" t="s">
+    <row r="235" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A235" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="B208" s="3" t="s">
+      <c r="B235" s="3" t="s">
         <v>415</v>
       </c>
     </row>
-    <row r="209">
-      <c r="A209" s="1" t="s">
+    <row r="236" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A236" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="B209" s="3" t="s">
+      <c r="B236" s="3" t="s">
         <v>417</v>
       </c>
     </row>
-    <row r="210">
-      <c r="A210" s="1" t="s">
+    <row r="237" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A237" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="B210" s="3" t="s">
+      <c r="B237" s="3" t="s">
         <v>419</v>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="1" t="s">
+    <row r="238" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A238" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="B211" s="3" t="s">
+      <c r="B238" s="3" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="212">
-      <c r="A212" s="1" t="s">
+    <row r="239" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A239" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="B212" s="3" t="s">
+      <c r="B239" s="3" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="213">
-      <c r="A213" s="1" t="s">
+    <row r="240" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A240" s="1" t="s">
         <v>424</v>
       </c>
-      <c r="B213" s="3" t="s">
+      <c r="B240" s="3" t="s">
         <v>425</v>
       </c>
     </row>
-    <row r="214">
-      <c r="A214" s="1" t="s">
+    <row r="241" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A241" s="1" t="s">
         <v>426</v>
       </c>
-      <c r="B214" s="3" t="s">
+      <c r="B241" s="3" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="215">
-      <c r="A215" s="1" t="s">
+    <row r="242" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A242" s="1" t="s">
+        <v>492</v>
+      </c>
+      <c r="B242" s="3" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="243" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A243" s="1" t="s">
         <v>428</v>
       </c>
-      <c r="B215" s="3" t="s">
+      <c r="B243" s="3" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="216">
-      <c r="A216" s="1" t="s">
+    <row r="244" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A244" s="1" t="s">
         <v>430</v>
       </c>
-      <c r="B216" s="3" t="s">
+      <c r="B244" s="3" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="217">
-      <c r="A217" s="1" t="s">
+    <row r="245" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A245" s="1" t="s">
         <v>432</v>
       </c>
-      <c r="B217" s="3" t="s">
+      <c r="B245" s="3" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="218">
-      <c r="A218" s="1" t="s">
+    <row r="246" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A246" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="B218" s="3" t="s">
+      <c r="B246" s="3" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="219">
-      <c r="A219" s="1" t="s">
+    <row r="247" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A247" s="1" t="s">
         <v>436</v>
       </c>
-      <c r="B219" s="3" t="s">
+      <c r="B247" s="3" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="220">
-      <c r="A220" s="1" t="s">
+    <row r="248" spans="1:2" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A248" s="1" t="s">
         <v>438</v>
       </c>
-      <c r="B220" s="3" t="s">
+      <c r="B248" s="3" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="221">
-      <c r="A221" s="1" t="s">
-        <v>440</v>
-      </c>
-      <c r="B221" s="3" t="s">
-        <v>441</v>
+    <row r="249" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A249" s="1" t="s">
+        <v>494</v>
+      </c>
+      <c r="B249" s="4" t="s">
+        <v>495</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B1"/>
-    <hyperlink r:id="rId2" ref="B2"/>
-    <hyperlink r:id="rId3" ref="B3"/>
-    <hyperlink r:id="rId4" ref="B4"/>
-    <hyperlink r:id="rId5" ref="B5"/>
-    <hyperlink r:id="rId6" ref="B6"/>
-    <hyperlink r:id="rId7" ref="B7"/>
-    <hyperlink r:id="rId8" ref="B8"/>
-    <hyperlink r:id="rId9" ref="B9"/>
-    <hyperlink r:id="rId10" ref="B10"/>
-    <hyperlink r:id="rId11" ref="B11"/>
-    <hyperlink r:id="rId12" ref="B12"/>
-    <hyperlink r:id="rId13" ref="B13"/>
-    <hyperlink r:id="rId14" ref="B14"/>
-    <hyperlink r:id="rId15" ref="B15"/>
-    <hyperlink r:id="rId16" ref="B16"/>
-    <hyperlink r:id="rId17" ref="B17"/>
-    <hyperlink r:id="rId18" ref="B18"/>
-    <hyperlink r:id="rId19" ref="B19"/>
-    <hyperlink r:id="rId20" ref="B20"/>
-    <hyperlink r:id="rId21" ref="B21"/>
-    <hyperlink r:id="rId22" ref="B22"/>
-    <hyperlink r:id="rId23" ref="B23"/>
-    <hyperlink r:id="rId24" ref="B24"/>
-    <hyperlink r:id="rId25" ref="B25"/>
-    <hyperlink r:id="rId26" ref="B26"/>
-    <hyperlink r:id="rId27" ref="B27"/>
-    <hyperlink r:id="rId28" ref="B28"/>
-    <hyperlink r:id="rId29" ref="B29"/>
-    <hyperlink r:id="rId30" ref="B30"/>
-    <hyperlink r:id="rId31" ref="B31"/>
-    <hyperlink r:id="rId32" ref="B32"/>
-    <hyperlink r:id="rId33" ref="B33"/>
-    <hyperlink r:id="rId34" ref="B34"/>
-    <hyperlink r:id="rId35" ref="B35"/>
-    <hyperlink r:id="rId36" ref="B36"/>
-    <hyperlink r:id="rId37" ref="B37"/>
-    <hyperlink r:id="rId38" ref="B38"/>
-    <hyperlink r:id="rId39" ref="B39"/>
-    <hyperlink r:id="rId40" ref="B40"/>
-    <hyperlink r:id="rId41" ref="B41"/>
-    <hyperlink r:id="rId42" ref="B42"/>
-    <hyperlink r:id="rId43" ref="B43"/>
-    <hyperlink r:id="rId44" ref="B44"/>
-    <hyperlink r:id="rId45" ref="B45"/>
-    <hyperlink r:id="rId46" ref="B46"/>
-    <hyperlink r:id="rId47" ref="B47"/>
-    <hyperlink r:id="rId48" ref="B48"/>
-    <hyperlink r:id="rId49" ref="B49"/>
-    <hyperlink r:id="rId50" ref="B50"/>
-    <hyperlink r:id="rId51" ref="B51"/>
-    <hyperlink r:id="rId52" ref="B52"/>
-    <hyperlink r:id="rId53" ref="B53"/>
-    <hyperlink r:id="rId54" ref="B54"/>
-    <hyperlink r:id="rId55" ref="B55"/>
-    <hyperlink r:id="rId56" ref="B56"/>
-    <hyperlink r:id="rId57" ref="B57"/>
-    <hyperlink r:id="rId58" ref="B58"/>
-    <hyperlink r:id="rId59" ref="B59"/>
-    <hyperlink r:id="rId60" ref="B60"/>
-    <hyperlink r:id="rId61" ref="B61"/>
-    <hyperlink r:id="rId62" ref="B62"/>
-    <hyperlink r:id="rId63" ref="B63"/>
-    <hyperlink r:id="rId64" ref="B64"/>
-    <hyperlink r:id="rId65" ref="B65"/>
-    <hyperlink r:id="rId66" ref="B66"/>
-    <hyperlink r:id="rId67" ref="B67"/>
-    <hyperlink r:id="rId68" ref="B68"/>
-    <hyperlink r:id="rId69" ref="B69"/>
-    <hyperlink r:id="rId70" ref="B70"/>
-    <hyperlink r:id="rId71" ref="B71"/>
-    <hyperlink r:id="rId72" ref="B72"/>
-    <hyperlink r:id="rId73" ref="B73"/>
-    <hyperlink r:id="rId74" ref="B74"/>
-    <hyperlink r:id="rId75" ref="B75"/>
-    <hyperlink r:id="rId76" ref="B76"/>
-    <hyperlink r:id="rId77" ref="B77"/>
-    <hyperlink r:id="rId78" ref="B78"/>
-    <hyperlink r:id="rId79" ref="B79"/>
-    <hyperlink r:id="rId80" ref="B80"/>
-    <hyperlink r:id="rId81" ref="B81"/>
-    <hyperlink r:id="rId82" ref="B82"/>
-    <hyperlink r:id="rId83" ref="B83"/>
-    <hyperlink r:id="rId84" ref="B84"/>
-    <hyperlink r:id="rId85" ref="B85"/>
-    <hyperlink r:id="rId86" ref="B86"/>
-    <hyperlink r:id="rId87" ref="B87"/>
-    <hyperlink r:id="rId88" ref="B88"/>
-    <hyperlink r:id="rId89" ref="B89"/>
-    <hyperlink r:id="rId90" ref="B90"/>
-    <hyperlink r:id="rId91" ref="B91"/>
-    <hyperlink r:id="rId92" ref="B92"/>
-    <hyperlink r:id="rId93" ref="B93"/>
-    <hyperlink r:id="rId94" ref="B94"/>
-    <hyperlink r:id="rId95" ref="B95"/>
-    <hyperlink r:id="rId96" ref="B96"/>
-    <hyperlink r:id="rId97" ref="B97"/>
-    <hyperlink r:id="rId98" ref="B98"/>
-    <hyperlink r:id="rId99" ref="B99"/>
-    <hyperlink r:id="rId100" ref="B100"/>
-    <hyperlink r:id="rId101" ref="B101"/>
-    <hyperlink r:id="rId102" ref="B102"/>
-    <hyperlink r:id="rId103" ref="B103"/>
-    <hyperlink r:id="rId104" ref="B104"/>
-    <hyperlink r:id="rId105" ref="B105"/>
-    <hyperlink r:id="rId106" ref="B106"/>
-    <hyperlink r:id="rId107" ref="B107"/>
-    <hyperlink r:id="rId108" ref="B108"/>
-    <hyperlink r:id="rId109" ref="B109"/>
-    <hyperlink r:id="rId110" ref="B110"/>
-    <hyperlink r:id="rId111" ref="B111"/>
-    <hyperlink r:id="rId112" ref="B112"/>
-    <hyperlink r:id="rId113" ref="B113"/>
-    <hyperlink r:id="rId114" ref="B114"/>
-    <hyperlink r:id="rId115" ref="B115"/>
-    <hyperlink r:id="rId116" ref="B116"/>
-    <hyperlink r:id="rId117" ref="B117"/>
-    <hyperlink r:id="rId118" ref="B118"/>
-    <hyperlink r:id="rId119" ref="B119"/>
-    <hyperlink r:id="rId120" ref="B120"/>
-    <hyperlink r:id="rId121" ref="B121"/>
-    <hyperlink r:id="rId122" ref="B122"/>
-    <hyperlink r:id="rId123" ref="B123"/>
-    <hyperlink r:id="rId124" ref="B124"/>
-    <hyperlink r:id="rId125" ref="B125"/>
-    <hyperlink r:id="rId126" ref="B126"/>
-    <hyperlink r:id="rId127" ref="B127"/>
-    <hyperlink r:id="rId128" ref="B128"/>
-    <hyperlink r:id="rId129" ref="B129"/>
-    <hyperlink r:id="rId130" ref="B130"/>
-    <hyperlink r:id="rId131" ref="B131"/>
-    <hyperlink r:id="rId132" ref="B132"/>
-    <hyperlink r:id="rId133" ref="B133"/>
-    <hyperlink r:id="rId134" ref="B134"/>
-    <hyperlink r:id="rId135" ref="B135"/>
-    <hyperlink r:id="rId136" ref="B136"/>
-    <hyperlink r:id="rId137" ref="B137"/>
-    <hyperlink r:id="rId138" ref="B138"/>
-    <hyperlink r:id="rId139" ref="B139"/>
-    <hyperlink r:id="rId140" ref="B140"/>
-    <hyperlink r:id="rId141" ref="B141"/>
-    <hyperlink r:id="rId142" ref="B142"/>
-    <hyperlink r:id="rId143" ref="B143"/>
-    <hyperlink r:id="rId144" ref="B144"/>
-    <hyperlink r:id="rId145" ref="B145"/>
-    <hyperlink r:id="rId146" ref="B146"/>
-    <hyperlink r:id="rId147" ref="B147"/>
-    <hyperlink r:id="rId148" ref="B148"/>
-    <hyperlink r:id="rId149" ref="B149"/>
-    <hyperlink r:id="rId150" ref="B150"/>
-    <hyperlink r:id="rId151" ref="B151"/>
-    <hyperlink r:id="rId152" ref="B152"/>
-    <hyperlink r:id="rId153" ref="B153"/>
-    <hyperlink r:id="rId154" ref="B154"/>
-    <hyperlink r:id="rId155" ref="B155"/>
-    <hyperlink r:id="rId156" ref="B156"/>
-    <hyperlink r:id="rId157" ref="B157"/>
-    <hyperlink r:id="rId158" ref="B158"/>
-    <hyperlink r:id="rId159" ref="B159"/>
-    <hyperlink r:id="rId160" ref="B160"/>
-    <hyperlink r:id="rId161" ref="B161"/>
-    <hyperlink r:id="rId162" ref="B162"/>
-    <hyperlink r:id="rId163" ref="B163"/>
-    <hyperlink r:id="rId164" ref="B164"/>
-    <hyperlink r:id="rId165" ref="B165"/>
-    <hyperlink r:id="rId166" ref="B166"/>
-    <hyperlink r:id="rId167" ref="B167"/>
-    <hyperlink r:id="rId168" ref="B168"/>
-    <hyperlink r:id="rId169" ref="B169"/>
-    <hyperlink r:id="rId170" ref="B170"/>
-    <hyperlink r:id="rId171" ref="B171"/>
-    <hyperlink r:id="rId172" ref="B172"/>
-    <hyperlink r:id="rId173" ref="B173"/>
-    <hyperlink r:id="rId174" ref="B174"/>
-    <hyperlink r:id="rId175" ref="B175"/>
-    <hyperlink r:id="rId176" ref="B176"/>
-    <hyperlink r:id="rId177" ref="B177"/>
-    <hyperlink r:id="rId178" ref="B178"/>
-    <hyperlink r:id="rId179" ref="B179"/>
-    <hyperlink r:id="rId180" ref="B180"/>
-    <hyperlink r:id="rId181" ref="B181"/>
-    <hyperlink r:id="rId182" ref="B182"/>
-    <hyperlink r:id="rId183" ref="B183"/>
-    <hyperlink r:id="rId184" ref="B184"/>
-    <hyperlink r:id="rId185" ref="B185"/>
-    <hyperlink r:id="rId186" ref="B186"/>
-    <hyperlink r:id="rId187" ref="B187"/>
-    <hyperlink r:id="rId188" ref="B188"/>
-    <hyperlink r:id="rId189" ref="B189"/>
-    <hyperlink r:id="rId190" ref="B190"/>
-    <hyperlink r:id="rId191" ref="B191"/>
-    <hyperlink r:id="rId192" ref="B192"/>
-    <hyperlink r:id="rId193" ref="B193"/>
-    <hyperlink r:id="rId194" ref="B194"/>
-    <hyperlink r:id="rId195" ref="B195"/>
-    <hyperlink r:id="rId196" ref="B196"/>
-    <hyperlink r:id="rId197" ref="B197"/>
-    <hyperlink r:id="rId198" ref="B198"/>
-    <hyperlink r:id="rId199" ref="B199"/>
-    <hyperlink r:id="rId200" ref="B200"/>
-    <hyperlink r:id="rId201" ref="B201"/>
-    <hyperlink r:id="rId202" ref="B202"/>
-    <hyperlink r:id="rId203" ref="B203"/>
-    <hyperlink r:id="rId204" ref="B204"/>
-    <hyperlink r:id="rId205" ref="B205"/>
-    <hyperlink r:id="rId206" ref="B206"/>
-    <hyperlink r:id="rId207" ref="B207"/>
-    <hyperlink r:id="rId208" ref="B208"/>
-    <hyperlink r:id="rId209" ref="B209"/>
-    <hyperlink r:id="rId210" ref="B210"/>
-    <hyperlink r:id="rId211" ref="B211"/>
-    <hyperlink r:id="rId212" ref="B212"/>
-    <hyperlink r:id="rId213" ref="B213"/>
-    <hyperlink r:id="rId214" ref="B214"/>
-    <hyperlink r:id="rId215" ref="B215"/>
-    <hyperlink r:id="rId216" ref="B216"/>
-    <hyperlink r:id="rId217" ref="B217"/>
-    <hyperlink r:id="rId218" ref="B218"/>
-    <hyperlink r:id="rId219" ref="B219"/>
-    <hyperlink r:id="rId220" ref="B220"/>
-    <hyperlink r:id="rId221" ref="B221"/>
+    <hyperlink ref="B1" r:id="rId1"/>
+    <hyperlink ref="B2" r:id="rId2"/>
+    <hyperlink ref="B3" r:id="rId3"/>
+    <hyperlink ref="B4" r:id="rId4"/>
+    <hyperlink ref="B5" r:id="rId5"/>
+    <hyperlink ref="B6" r:id="rId6"/>
+    <hyperlink ref="B7" r:id="rId7"/>
+    <hyperlink ref="B8" r:id="rId8"/>
+    <hyperlink ref="B9" r:id="rId9"/>
+    <hyperlink ref="B10" r:id="rId10"/>
+    <hyperlink ref="B11" r:id="rId11"/>
+    <hyperlink ref="B12" r:id="rId12"/>
+    <hyperlink ref="B13" r:id="rId13"/>
+    <hyperlink ref="B14" r:id="rId14"/>
+    <hyperlink ref="B15" r:id="rId15"/>
+    <hyperlink ref="B16" r:id="rId16"/>
+    <hyperlink ref="B17" r:id="rId17"/>
+    <hyperlink ref="B18" r:id="rId18"/>
+    <hyperlink ref="B20" r:id="rId19"/>
+    <hyperlink ref="B21" r:id="rId20"/>
+    <hyperlink ref="B22" r:id="rId21"/>
+    <hyperlink ref="B23" r:id="rId22"/>
+    <hyperlink ref="B24" r:id="rId23"/>
+    <hyperlink ref="B25" r:id="rId24"/>
+    <hyperlink ref="B26" r:id="rId25"/>
+    <hyperlink ref="B27" r:id="rId26"/>
+    <hyperlink ref="B28" r:id="rId27"/>
+    <hyperlink ref="B29" r:id="rId28"/>
+    <hyperlink ref="B30" r:id="rId29"/>
+    <hyperlink ref="B31" r:id="rId30"/>
+    <hyperlink ref="B32" r:id="rId31"/>
+    <hyperlink ref="B33" r:id="rId32"/>
+    <hyperlink ref="B34" r:id="rId33"/>
+    <hyperlink ref="B35" r:id="rId34"/>
+    <hyperlink ref="B36" r:id="rId35"/>
+    <hyperlink ref="B37" r:id="rId36"/>
+    <hyperlink ref="B38" r:id="rId37"/>
+    <hyperlink ref="B39" r:id="rId38"/>
+    <hyperlink ref="B40" r:id="rId39"/>
+    <hyperlink ref="B41" r:id="rId40"/>
+    <hyperlink ref="B42" r:id="rId41"/>
+    <hyperlink ref="B43" r:id="rId42"/>
+    <hyperlink ref="B44" r:id="rId43"/>
+    <hyperlink ref="B45" r:id="rId44"/>
+    <hyperlink ref="B46" r:id="rId45"/>
+    <hyperlink ref="B47" r:id="rId46"/>
+    <hyperlink ref="B48" r:id="rId47"/>
+    <hyperlink ref="B49" r:id="rId48"/>
+    <hyperlink ref="B50" r:id="rId49"/>
+    <hyperlink ref="B51" r:id="rId50"/>
+    <hyperlink ref="B52" r:id="rId51"/>
+    <hyperlink ref="B53" r:id="rId52"/>
+    <hyperlink ref="B54" r:id="rId53"/>
+    <hyperlink ref="B55" r:id="rId54"/>
+    <hyperlink ref="B56" r:id="rId55"/>
+    <hyperlink ref="B58" r:id="rId56"/>
+    <hyperlink ref="B59" r:id="rId57"/>
+    <hyperlink ref="B60" r:id="rId58"/>
+    <hyperlink ref="B61" r:id="rId59"/>
+    <hyperlink ref="B62" r:id="rId60"/>
+    <hyperlink ref="B63" r:id="rId61"/>
+    <hyperlink ref="B64" r:id="rId62"/>
+    <hyperlink ref="B65" r:id="rId63"/>
+    <hyperlink ref="B66" r:id="rId64"/>
+    <hyperlink ref="B67" r:id="rId65"/>
+    <hyperlink ref="B68" r:id="rId66"/>
+    <hyperlink ref="B69" r:id="rId67"/>
+    <hyperlink ref="B70" r:id="rId68"/>
+    <hyperlink ref="B71" r:id="rId69"/>
+    <hyperlink ref="B72" r:id="rId70"/>
+    <hyperlink ref="B73" r:id="rId71"/>
+    <hyperlink ref="B74" r:id="rId72"/>
+    <hyperlink ref="B75" r:id="rId73"/>
+    <hyperlink ref="B78" r:id="rId74"/>
+    <hyperlink ref="B79" r:id="rId75"/>
+    <hyperlink ref="B80" r:id="rId76"/>
+    <hyperlink ref="B81" r:id="rId77"/>
+    <hyperlink ref="B82" r:id="rId78"/>
+    <hyperlink ref="B83" r:id="rId79"/>
+    <hyperlink ref="B84" r:id="rId80"/>
+    <hyperlink ref="B85" r:id="rId81"/>
+    <hyperlink ref="B86" r:id="rId82"/>
+    <hyperlink ref="B87" r:id="rId83"/>
+    <hyperlink ref="B88" r:id="rId84"/>
+    <hyperlink ref="B89" r:id="rId85"/>
+    <hyperlink ref="B90" r:id="rId86"/>
+    <hyperlink ref="B91" r:id="rId87"/>
+    <hyperlink ref="B92" r:id="rId88"/>
+    <hyperlink ref="B93" r:id="rId89"/>
+    <hyperlink ref="B94" r:id="rId90"/>
+    <hyperlink ref="B95" r:id="rId91"/>
+    <hyperlink ref="B96" r:id="rId92"/>
+    <hyperlink ref="B97" r:id="rId93"/>
+    <hyperlink ref="B98" r:id="rId94"/>
+    <hyperlink ref="B99" r:id="rId95"/>
+    <hyperlink ref="B105" r:id="rId96"/>
+    <hyperlink ref="B106" r:id="rId97"/>
+    <hyperlink ref="B107" r:id="rId98"/>
+    <hyperlink ref="B108" r:id="rId99"/>
+    <hyperlink ref="B109" r:id="rId100"/>
+    <hyperlink ref="B110" r:id="rId101"/>
+    <hyperlink ref="B111" r:id="rId102"/>
+    <hyperlink ref="B112" r:id="rId103"/>
+    <hyperlink ref="B113" r:id="rId104"/>
+    <hyperlink ref="B114" r:id="rId105"/>
+    <hyperlink ref="B115" r:id="rId106"/>
+    <hyperlink ref="B116" r:id="rId107"/>
+    <hyperlink ref="B117" r:id="rId108"/>
+    <hyperlink ref="B118" r:id="rId109"/>
+    <hyperlink ref="B119" r:id="rId110"/>
+    <hyperlink ref="B120" r:id="rId111"/>
+    <hyperlink ref="B121" r:id="rId112"/>
+    <hyperlink ref="B122" r:id="rId113"/>
+    <hyperlink ref="B125" r:id="rId114"/>
+    <hyperlink ref="B126" r:id="rId115"/>
+    <hyperlink ref="B127" r:id="rId116"/>
+    <hyperlink ref="B128" r:id="rId117"/>
+    <hyperlink ref="B129" r:id="rId118"/>
+    <hyperlink ref="B130" r:id="rId119"/>
+    <hyperlink ref="B132" r:id="rId120"/>
+    <hyperlink ref="B135" r:id="rId121"/>
+    <hyperlink ref="B136" r:id="rId122"/>
+    <hyperlink ref="B139" r:id="rId123"/>
+    <hyperlink ref="B140" r:id="rId124"/>
+    <hyperlink ref="B141" r:id="rId125"/>
+    <hyperlink ref="B142" r:id="rId126"/>
+    <hyperlink ref="B143" r:id="rId127"/>
+    <hyperlink ref="B144" r:id="rId128"/>
+    <hyperlink ref="B146" r:id="rId129"/>
+    <hyperlink ref="B147" r:id="rId130"/>
+    <hyperlink ref="B148" r:id="rId131"/>
+    <hyperlink ref="B149" r:id="rId132"/>
+    <hyperlink ref="B150" r:id="rId133"/>
+    <hyperlink ref="B151" r:id="rId134"/>
+    <hyperlink ref="B152" r:id="rId135"/>
+    <hyperlink ref="B153" r:id="rId136"/>
+    <hyperlink ref="B154" r:id="rId137"/>
+    <hyperlink ref="B155" r:id="rId138"/>
+    <hyperlink ref="B156" r:id="rId139"/>
+    <hyperlink ref="B157" r:id="rId140"/>
+    <hyperlink ref="B158" r:id="rId141"/>
+    <hyperlink ref="B159" r:id="rId142"/>
+    <hyperlink ref="B160" r:id="rId143"/>
+    <hyperlink ref="B161" r:id="rId144"/>
+    <hyperlink ref="B162" r:id="rId145"/>
+    <hyperlink ref="B165" r:id="rId146"/>
+    <hyperlink ref="B166" r:id="rId147"/>
+    <hyperlink ref="B167" r:id="rId148"/>
+    <hyperlink ref="B168" r:id="rId149"/>
+    <hyperlink ref="B172" r:id="rId150"/>
+    <hyperlink ref="B173" r:id="rId151"/>
+    <hyperlink ref="B174" r:id="rId152"/>
+    <hyperlink ref="B175" r:id="rId153"/>
+    <hyperlink ref="B176" r:id="rId154"/>
+    <hyperlink ref="B178" r:id="rId155"/>
+    <hyperlink ref="B179" r:id="rId156"/>
+    <hyperlink ref="B180" r:id="rId157"/>
+    <hyperlink ref="B181" r:id="rId158"/>
+    <hyperlink ref="B182" r:id="rId159"/>
+    <hyperlink ref="B183" r:id="rId160"/>
+    <hyperlink ref="B184" r:id="rId161"/>
+    <hyperlink ref="B185" r:id="rId162"/>
+    <hyperlink ref="B186" r:id="rId163"/>
+    <hyperlink ref="B187" r:id="rId164"/>
+    <hyperlink ref="B191" r:id="rId165"/>
+    <hyperlink ref="B192" r:id="rId166"/>
+    <hyperlink ref="B193" r:id="rId167"/>
+    <hyperlink ref="B194" r:id="rId168"/>
+    <hyperlink ref="B195" r:id="rId169"/>
+    <hyperlink ref="B196" r:id="rId170"/>
+    <hyperlink ref="B197" r:id="rId171"/>
+    <hyperlink ref="B198" r:id="rId172"/>
+    <hyperlink ref="B199" r:id="rId173"/>
+    <hyperlink ref="B200" r:id="rId174"/>
+    <hyperlink ref="B201" r:id="rId175"/>
+    <hyperlink ref="B202" r:id="rId176"/>
+    <hyperlink ref="B203" r:id="rId177"/>
+    <hyperlink ref="B204" r:id="rId178"/>
+    <hyperlink ref="B205" r:id="rId179"/>
+    <hyperlink ref="B206" r:id="rId180"/>
+    <hyperlink ref="B207" r:id="rId181"/>
+    <hyperlink ref="B208" r:id="rId182"/>
+    <hyperlink ref="B209" r:id="rId183"/>
+    <hyperlink ref="B210" r:id="rId184"/>
+    <hyperlink ref="B211" r:id="rId185"/>
+    <hyperlink ref="B212" r:id="rId186"/>
+    <hyperlink ref="B213" r:id="rId187"/>
+    <hyperlink ref="B214" r:id="rId188"/>
+    <hyperlink ref="B215" r:id="rId189"/>
+    <hyperlink ref="B216" r:id="rId190"/>
+    <hyperlink ref="B217" r:id="rId191"/>
+    <hyperlink ref="B218" r:id="rId192"/>
+    <hyperlink ref="B219" r:id="rId193"/>
+    <hyperlink ref="B220" r:id="rId194"/>
+    <hyperlink ref="B221" r:id="rId195"/>
+    <hyperlink ref="B222" r:id="rId196"/>
+    <hyperlink ref="B223" r:id="rId197"/>
+    <hyperlink ref="B224" r:id="rId198"/>
+    <hyperlink ref="B225" r:id="rId199"/>
+    <hyperlink ref="B226" r:id="rId200"/>
+    <hyperlink ref="B227" r:id="rId201"/>
+    <hyperlink ref="B228" r:id="rId202"/>
+    <hyperlink ref="B229" r:id="rId203"/>
+    <hyperlink ref="B230" r:id="rId204"/>
+    <hyperlink ref="B231" r:id="rId205"/>
+    <hyperlink ref="B232" r:id="rId206"/>
+    <hyperlink ref="B233" r:id="rId207"/>
+    <hyperlink ref="B234" r:id="rId208"/>
+    <hyperlink ref="B235" r:id="rId209"/>
+    <hyperlink ref="B236" r:id="rId210"/>
+    <hyperlink ref="B237" r:id="rId211"/>
+    <hyperlink ref="B238" r:id="rId212"/>
+    <hyperlink ref="B239" r:id="rId213"/>
+    <hyperlink ref="B240" r:id="rId214"/>
+    <hyperlink ref="B241" r:id="rId215"/>
+    <hyperlink ref="B243" r:id="rId216"/>
+    <hyperlink ref="B244" r:id="rId217"/>
+    <hyperlink ref="B245" r:id="rId218"/>
+    <hyperlink ref="B246" r:id="rId219"/>
+    <hyperlink ref="B247" r:id="rId220"/>
+    <hyperlink ref="B248" r:id="rId221"/>
+    <hyperlink ref="B249" r:id="rId222"/>
   </hyperlinks>
-  <drawing r:id="rId222"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId223"/>
 </worksheet>
 </file>
</xml_diff>